<commit_message>
feat: add group formation and management feature with real-time support
</commit_message>
<xml_diff>
--- a/server/DS_Mentor_email.xlsx
+++ b/server/DS_Mentor_email.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\project\exe\server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D895E99F-7A0D-4B77-B334-4922F5907D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A1B173B-4F0B-483B-B84B-BBE60E215458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5157" uniqueCount="2342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5159" uniqueCount="2344">
   <si>
     <t>GroupName</t>
   </si>
@@ -7057,10 +7057,16 @@
     <t>CS190452</t>
   </si>
   <si>
+    <t>djnd</t>
+  </si>
+  <si>
+    <t>voanhbendjndnd@gmail.com</t>
+  </si>
+  <si>
+    <t>misaka</t>
+  </si>
+  <si>
     <t>voanhben111@gmail.com</t>
-  </si>
-  <si>
-    <t>trang</t>
   </si>
 </sst>
 </file>
@@ -7080,7 +7086,15 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
     </font>
@@ -7093,15 +7107,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="163"/>
     </font>
@@ -7127,13 +7133,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC0E6F5"/>
+        <fgColor rgb="FFCAEDFB"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFCAEDFB"/>
+        <fgColor rgb="FFC0E6F5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -7170,7 +7176,7 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
@@ -7184,23 +7190,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -25902,38 +25908,50 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8403D725-964A-41D0-8E58-9A354E36CA30}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="19.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.109375" style="5" customWidth="1"/>
-    <col min="2" max="2" width="22.109375" style="4" customWidth="1"/>
-    <col min="3" max="3" width="27.44140625" style="4" customWidth="1"/>
-    <col min="4" max="16384" width="19.88671875" style="5"/>
+    <col min="1" max="1" width="7.109375" style="7" customWidth="1"/>
+    <col min="2" max="2" width="22.109375" style="9" customWidth="1"/>
+    <col min="3" max="3" width="27.44140625" style="9" customWidth="1"/>
+    <col min="4" max="16384" width="19.88671875" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="9"/>
-      <c r="B1" s="6" t="s">
+      <c r="A1" s="4"/>
+      <c r="B1" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="9">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="8" t="s">
+        <v>2340</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>2341</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>2340</v>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>2342</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>2343</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{AE987024-25C6-48D1-A252-A73471C60A6E}"/>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{14E9D22C-F6B5-4BD9-9D70-9AEEDC41C0C1}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{FDC32AE0-5942-4745-8EF1-07AEA6AB4DE1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: initialize full-stack project structure with student, lecturer, and deadline management modules
</commit_message>
<xml_diff>
--- a/server/DS_Mentor_email.xlsx
+++ b/server/DS_Mentor_email.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\project\exe\server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A1B173B-4F0B-483B-B84B-BBE60E215458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D895E99F-7A0D-4B77-B334-4922F5907D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5159" uniqueCount="2344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5157" uniqueCount="2342">
   <si>
     <t>GroupName</t>
   </si>
@@ -7057,16 +7057,10 @@
     <t>CS190452</t>
   </si>
   <si>
-    <t>djnd</t>
-  </si>
-  <si>
-    <t>voanhbendjndnd@gmail.com</t>
-  </si>
-  <si>
-    <t>misaka</t>
-  </si>
-  <si>
     <t>voanhben111@gmail.com</t>
+  </si>
+  <si>
+    <t>trang</t>
   </si>
 </sst>
 </file>
@@ -7086,15 +7080,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="163"/>
     </font>
@@ -7107,7 +7093,15 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
     </font>
@@ -7133,13 +7127,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFCAEDFB"/>
+        <fgColor rgb="FFC0E6F5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC0E6F5"/>
+        <fgColor rgb="FFCAEDFB"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -7176,7 +7170,7 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
@@ -7190,23 +7184,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -25908,50 +25902,38 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8403D725-964A-41D0-8E58-9A354E36CA30}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultColWidth="19.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.109375" style="7" customWidth="1"/>
-    <col min="2" max="2" width="22.109375" style="9" customWidth="1"/>
-    <col min="3" max="3" width="27.44140625" style="9" customWidth="1"/>
-    <col min="4" max="16384" width="19.88671875" style="7"/>
+    <col min="1" max="1" width="7.109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="22.109375" style="4" customWidth="1"/>
+    <col min="3" max="3" width="27.44140625" style="4" customWidth="1"/>
+    <col min="4" max="16384" width="19.88671875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="4"/>
-      <c r="B1" s="5" t="s">
+      <c r="A1" s="9"/>
+      <c r="B1" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="4">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="8" t="s">
+        <v>2341</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>2340</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>2341</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="4">
-        <v>2</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>2342</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>2343</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{14E9D22C-F6B5-4BD9-9D70-9AEEDC41C0C1}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{FDC32AE0-5942-4745-8EF1-07AEA6AB4DE1}"/>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{AE987024-25C6-48D1-A252-A73471C60A6E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>